<commit_message>
style(lead-magnets): format all documents to 100% NASKAH.FK standard (Times New Roman, Open-Table, 4-4-3-3 margins)
</commit_message>
<xml_diff>
--- a/07_LEAD_MAGNETS/01_DIAGNOSIS_Kalkulator_Tabel_2x2_Naskah.xlsx
+++ b/07_LEAD_MAGNETS/01_DIAGNOSIS_Kalkulator_Tabel_2x2_Naskah.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,60 +29,42 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <color rgb="00000000"/>
+      <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <i val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00555555"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="00071726"/>
+      <color rgb="00000000"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00071726"/>
+      <name val="Times New Roman"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00E85929"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001D2939"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00E85929"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <i val="1"/>
-      <color rgb="00071726"/>
+      <color rgb="00333333"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -91,36 +73,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00071726"/>
-        <bgColor rgb="00071726"/>
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDF4EB"/>
-        <bgColor rgb="00FDF4EB"/>
+        <fgColor rgb="00EAEAEA"/>
+        <bgColor rgb="00EAEAEA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBF3FA"/>
-        <bgColor rgb="00EBF3FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0F4F8"/>
-        <bgColor rgb="00F0F4F8"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -129,82 +99,92 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00D0D5DD"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D0D5DD"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D0D5DD"/>
+      <top style="medium">
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D0D5DD"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D0D5DD"/>
+        <color rgb="00CCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00D0D5DD"/>
+        <color rgb="00CCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00D0D5DD"/>
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
       </top>
       <bottom style="medium">
-        <color rgb="00071726"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -572,49 +552,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H26"/>
+  <dimension ref="B1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>KALKULATOR UJI DIAGNOSTIK TABEL 2x2 — NASKAH.FK</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Official Academic Companion — Masukkan angka pada sel berwarna KUNING. Hasil terhitung otomatis.</t>
+          <t>Standar Pelaporan Ilmiah Bab 4 Skripsi FK (Input data pada sel berwarna kuning)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>1. TABEL KONTINGENSI 2x2 (INPUT DATA)</t>
+          <t>1. Tabel Kontingensi 2x2 (Input Data Sampel)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>BAKU EMAS (GOLD STANDARD)</t>
+          <t>Baku Emas (Gold Standard)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>ALAT UJI BARU</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Alat Uji Baru</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -634,15 +614,15 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Positif (+)</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="8" t="n">
         <v>85</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E7" s="6">
@@ -651,15 +631,15 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Negatif (-)</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <v>90</v>
       </c>
       <c r="E8" s="6">
@@ -668,16 +648,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Total Baku Emas</t>
         </is>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="9">
         <f>C7+C8</f>
         <v/>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="9">
         <f>D7+D8</f>
         <v/>
       </c>
@@ -689,248 +669,248 @@
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2. HASIL PERHITUNGAN PARAMETER DIAGNOSTIK</t>
+          <t>2. Hasil Perhitungan Parameter Diagnostik</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Parameter Diagnostik</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Rumus Matematis</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Nilai Desimal</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Persentase (%)</t>
         </is>
       </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>Interpretasi Klinis untuk Naskah Skripsi</t>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Interpretasi Klinis Bab 4 Skripsi</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Sensitivitas (Sensitivity / True Positive Rate)</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>TP / (TP + FN)</t>
         </is>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="12">
         <f>C7/C9</f>
         <v/>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="13">
         <f>C7/C9</f>
         <v/>
       </c>
-      <c r="F13" s="15" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Kemampuan alat mendeteksi subjek yang benar-benar sakit.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Spesifisitas (Specificity / True Negative Rate)</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>TN / (TN + FP)</t>
         </is>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="12">
         <f>D8/D9</f>
         <v/>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="13">
         <f>D8/D9</f>
         <v/>
       </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Kemampuan alat menyaring subjek yang benar-benar sehat.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Nilai Prediktif Positif (PPV / Precision)</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>TP / (TP + FP)</t>
         </is>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="12">
         <f>C7/E7</f>
         <v/>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="13">
         <f>C7/E7</f>
         <v/>
       </c>
-      <c r="F15" s="15" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>Probabilitas subjek benar sakit jika hasil tes positif.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Nilai Prediktif Negatif (NPV)</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>TN / (TN + FN)</t>
         </is>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="12">
         <f>D8/E8</f>
         <v/>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="13">
         <f>D8/E8</f>
         <v/>
       </c>
-      <c r="F16" s="15" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>Probabilitas subjek benar sehat jika hasil tes negatif.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Akurasi Diagnostik (Accuracy)</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Akurasi Diagnostik (Diagnostic Accuracy)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>(TP + TN) / Total N</t>
         </is>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="12">
         <f>(C7+D8)/E9</f>
         <v/>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="13">
         <f>(C7+D8)/E9</f>
         <v/>
       </c>
-      <c r="F17" s="15" t="inlineStr">
-        <is>
-          <t>Proporsi keseluruhan diagnosis yang benar.</t>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Proporsi keseluruhan diagnosis yang terbukti benar.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Positive Likelihood Ratio (LR+)</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>Sensitivitas / (1 - Spesifisitas)</t>
         </is>
       </c>
-      <c r="D18" s="13">
+      <c r="D18" s="12">
         <f>(C7/C9)/(1-(D8/D9))</f>
         <v/>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F18" s="15" t="inlineStr">
-        <is>
-          <t>Rasio peningkatan kemungkinan sakit jika tes positif (&gt;10 = sangat kuat).</t>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Peningkatan kemungkinan sakit jika tes positif (&gt;10 = sangat baik).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Negative Likelihood Ratio (LR-)</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>(1 - Sensitivitas) / Spesifisitas</t>
         </is>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="12">
         <f>(1-(C7/C9))/(D8/D9)</f>
         <v/>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>Rasio penurunan kemungkinan sakit jika tes negatif (&lt;0.1 = sangat kuat).</t>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Penurunan kemungkinan sakit jika tes negatif (&lt;0.1 = sangat baik).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Prevalensi Penyakit (Pre-test Probability)</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>(TP + FN) / Total N</t>
         </is>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="18">
         <f>C9/E9</f>
         <v/>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="19">
         <f>C9/E9</f>
         <v/>
       </c>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>Proporsi populasi sakit berdasarkan baku emas.</t>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t>Proporsi subjek sakit berdasarkan baku emas.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>3. TEMPLATE KALIMAT PELAPORAN BAB 4 SKRIPSI FK (SIAP COPY)</t>
+          <t>3. Template Kalimat Pelaporan Bab 4 Skripsi FK</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="21" t="inlineStr">
         <is>
           <t>Berdasarkan hasil uji diagnostik terhadap total responden (N), diperoleh nilai sensitivitas alat sebesar [Persentase] dan spesifisitas sebesar [Persentase]. Nilai Prediktif Positif (PPV) tercatat sebesar [Persentase] dan Nilai Prediktif Negatif (NPV) sebesar [Persentase], dengan akurasi diagnostik keseluruhan mencapai [Persentase]. Nilai Positive Likelihood Ratio (LR+) sebesar [Nilai] menunjukkan kemampuan konfirmasi klinis yang memadai.</t>
         </is>
@@ -940,10 +920,10 @@
     <row r="26"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="C5:D5"/>
     <mergeCell ref="B24:F26"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="B1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>